<commit_message>
Correzione errori: [152,154,155,156,159,160,161,162,163,164,165,166,167,168,461,475] C004: È necessario NON valorizzare le colonne F, G, H, I poiché il caso di test non è applicabile [152,154,155,156,160,161,162,163] C012: È necessario NON valorizzare le seguenti colonne L
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#MYBUSINESSSOLUTIONSXX/MBS/INCARE/1.0/accreditamento-checklist_V8.3.0.xlsx
+++ b/GATEWAY/A1#111#MYBUSINESSSOLUTIONSXX/MBS/INCARE/1.0/accreditamento-checklist_V8.3.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\fse-middleware-accreditamento\GATEWAY\A1#111#MYBUSINESSSOLUTIONSXX\MBS\INCARE\1.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D629169C-4824-4ADF-8B58-16F10C0B5FEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BE27C4D-8639-47F4-A1FA-FD4249F75A51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1426" uniqueCount="587">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1418" uniqueCount="580">
   <si>
     <t>COME VALORIZZARE LA CHECKLIST (tab TestCases)</t>
   </si>
@@ -2100,18 +2100,6 @@
     <t>In questo caso il documento resta in coda di invio e verrà processato al successivo "round" del JOB. Da interfaccia è possibile effettuare lo start e lo stop dei servizi, e cofigurare la frequenza del JOB</t>
   </si>
   <si>
-    <t>Il sistema effettua l'uppercase del codice fiscale del paziente</t>
-  </si>
-  <si>
-    <t>Nel gestionale, la scheda paziente, è strutturata per selezionare la città di residenza (ed anche la città di domicilio) da una tendina, ed è un campo obbligatorio. Diversamente non può avvenire l'accettazione  e la refertazione</t>
-  </si>
-  <si>
-    <t>Nel gestionale, sia il nome che il cognome sono campi separati ed obbligatori per l'applicativo nella scheda paziente</t>
-  </si>
-  <si>
-    <t>Tendina a due valori</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Il gestionale non gestisce le ricette dei medici, e viene venduto solo a strutture che operano in regime </t>
     </r>
@@ -2125,15 +2113,6 @@
       </rPr>
       <t>NON CONVENZIONATO</t>
     </r>
-  </si>
-  <si>
-    <t>Nel gestionale, gli esami svolti dal paziente sono gestiti a carrello, con uno o più esami nel carrello. Non è possibile effettuare l'accettazione di un carrello senza nessuna prestazione, e non può il flusso andare avanti nella fase di generazione di un referto</t>
-  </si>
-  <si>
-    <t>In fase di scrittura del referto, il testo del referto è un campo obbligatorio</t>
-  </si>
-  <si>
-    <t>Dato non gestito dal gestionale. Il dottore scrive il quesito direttamente nel referto</t>
   </si>
   <si>
     <t>Dato non gestito dal gestionale. Il dottore scrive l’anamnesi patologica direttamente nel referto</t>
@@ -4309,7 +4288,7 @@
       </c>
       <c r="B2" s="48"/>
       <c r="C2" s="49" t="s">
-        <v>582</v>
+        <v>575</v>
       </c>
       <c r="D2" s="50"/>
       <c r="F2" s="6"/>
@@ -4337,7 +4316,7 @@
       </c>
       <c r="B3" s="52"/>
       <c r="C3" s="57" t="s">
-        <v>583</v>
+        <v>576</v>
       </c>
       <c r="D3" s="48"/>
       <c r="F3" s="6"/>
@@ -4363,7 +4342,7 @@
       <c r="A4" s="53"/>
       <c r="B4" s="54"/>
       <c r="C4" s="57" t="s">
-        <v>584</v>
+        <v>577</v>
       </c>
       <c r="D4" s="48"/>
       <c r="E4" s="4"/>
@@ -4390,7 +4369,7 @@
       <c r="A5" s="55"/>
       <c r="B5" s="56"/>
       <c r="C5" s="57" t="s">
-        <v>585</v>
+        <v>578</v>
       </c>
       <c r="D5" s="48"/>
       <c r="F5" s="6"/>
@@ -4734,7 +4713,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="33">
         <v>32</v>
       </c>
@@ -5056,7 +5035,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="33">
         <v>40</v>
       </c>
@@ -5386,7 +5365,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="31" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="33">
         <v>48</v>
       </c>
@@ -5420,7 +5399,7 @@
         <v>76</v>
       </c>
       <c r="O31" s="36" t="s">
-        <v>586</v>
+        <v>579</v>
       </c>
       <c r="P31" s="36" t="s">
         <v>76</v>
@@ -8573,9 +8552,7 @@
       <c r="E116" s="41" t="s">
         <v>247</v>
       </c>
-      <c r="F116" s="35">
-        <v>46095</v>
-      </c>
+      <c r="F116" s="35"/>
       <c r="G116" s="35"/>
       <c r="H116" s="35"/>
       <c r="I116" s="40"/>
@@ -8585,9 +8562,7 @@
       <c r="K116" s="36" t="s">
         <v>505</v>
       </c>
-      <c r="L116" s="36" t="s">
-        <v>554</v>
-      </c>
+      <c r="L116" s="36"/>
       <c r="M116" s="36"/>
       <c r="N116" s="36"/>
       <c r="O116" s="36"/>
@@ -8618,9 +8593,7 @@
       <c r="E117" s="41" t="s">
         <v>249</v>
       </c>
-      <c r="F117" s="35">
-        <v>46095</v>
-      </c>
+      <c r="F117" s="35"/>
       <c r="G117" s="35"/>
       <c r="H117" s="35"/>
       <c r="I117" s="40"/>
@@ -8630,9 +8603,7 @@
       <c r="K117" s="36" t="s">
         <v>504</v>
       </c>
-      <c r="L117" s="36" t="s">
-        <v>555</v>
-      </c>
+      <c r="L117" s="36"/>
       <c r="M117" s="36"/>
       <c r="N117" s="36"/>
       <c r="O117" s="36"/>
@@ -8663,9 +8634,7 @@
       <c r="E118" s="41" t="s">
         <v>251</v>
       </c>
-      <c r="F118" s="35">
-        <v>46095</v>
-      </c>
+      <c r="F118" s="35"/>
       <c r="G118" s="35"/>
       <c r="H118" s="35"/>
       <c r="I118" s="40"/>
@@ -8675,9 +8644,7 @@
       <c r="K118" s="36" t="s">
         <v>505</v>
       </c>
-      <c r="L118" s="36" t="s">
-        <v>556</v>
-      </c>
+      <c r="L118" s="36"/>
       <c r="M118" s="36"/>
       <c r="N118" s="36"/>
       <c r="O118" s="36"/>
@@ -8708,9 +8675,7 @@
       <c r="E119" s="41" t="s">
         <v>253</v>
       </c>
-      <c r="F119" s="35">
-        <v>46095</v>
-      </c>
+      <c r="F119" s="35"/>
       <c r="G119" s="35"/>
       <c r="H119" s="35"/>
       <c r="I119" s="40"/>
@@ -8720,9 +8685,7 @@
       <c r="K119" s="36" t="s">
         <v>504</v>
       </c>
-      <c r="L119" s="36" t="s">
-        <v>557</v>
-      </c>
+      <c r="L119" s="36"/>
       <c r="M119" s="36"/>
       <c r="N119" s="36"/>
       <c r="O119" s="36"/>
@@ -8753,9 +8716,7 @@
       <c r="E120" s="41" t="s">
         <v>255</v>
       </c>
-      <c r="F120" s="35">
-        <v>46095</v>
-      </c>
+      <c r="F120" s="35"/>
       <c r="G120" s="35"/>
       <c r="H120" s="35"/>
       <c r="I120" s="40"/>
@@ -8766,7 +8727,7 @@
         <v>506</v>
       </c>
       <c r="L120" s="36" t="s">
-        <v>558</v>
+        <v>554</v>
       </c>
       <c r="M120" s="36"/>
       <c r="N120" s="36"/>
@@ -8798,9 +8759,7 @@
       <c r="E121" s="41" t="s">
         <v>257</v>
       </c>
-      <c r="F121" s="35">
-        <v>46095</v>
-      </c>
+      <c r="F121" s="35"/>
       <c r="G121" s="35"/>
       <c r="H121" s="35"/>
       <c r="I121" s="40"/>
@@ -8810,9 +8769,7 @@
       <c r="K121" s="36" t="s">
         <v>505</v>
       </c>
-      <c r="L121" s="36" t="s">
-        <v>559</v>
-      </c>
+      <c r="L121" s="36"/>
       <c r="M121" s="36"/>
       <c r="N121" s="36"/>
       <c r="O121" s="36"/>
@@ -8843,9 +8800,7 @@
       <c r="E122" s="41" t="s">
         <v>259</v>
       </c>
-      <c r="F122" s="35">
-        <v>46095</v>
-      </c>
+      <c r="F122" s="35"/>
       <c r="G122" s="35"/>
       <c r="H122" s="35"/>
       <c r="I122" s="40"/>
@@ -8855,9 +8810,7 @@
       <c r="K122" s="36" t="s">
         <v>505</v>
       </c>
-      <c r="L122" s="36" t="s">
-        <v>560</v>
-      </c>
+      <c r="L122" s="36"/>
       <c r="M122" s="36"/>
       <c r="N122" s="36"/>
       <c r="O122" s="36"/>
@@ -8888,9 +8841,7 @@
       <c r="E123" s="41" t="s">
         <v>261</v>
       </c>
-      <c r="F123" s="35">
-        <v>46095</v>
-      </c>
+      <c r="F123" s="35"/>
       <c r="G123" s="35"/>
       <c r="H123" s="35"/>
       <c r="I123" s="40"/>
@@ -8900,9 +8851,7 @@
       <c r="K123" s="36" t="s">
         <v>502</v>
       </c>
-      <c r="L123" s="36" t="s">
-        <v>561</v>
-      </c>
+      <c r="L123" s="36"/>
       <c r="M123" s="36"/>
       <c r="N123" s="36"/>
       <c r="O123" s="36"/>
@@ -8933,9 +8882,7 @@
       <c r="E124" s="41" t="s">
         <v>263</v>
       </c>
-      <c r="F124" s="35">
-        <v>46095</v>
-      </c>
+      <c r="F124" s="35"/>
       <c r="G124" s="35"/>
       <c r="H124" s="35"/>
       <c r="I124" s="40"/>
@@ -8945,9 +8892,7 @@
       <c r="K124" s="36" t="s">
         <v>505</v>
       </c>
-      <c r="L124" s="36" t="s">
-        <v>559</v>
-      </c>
+      <c r="L124" s="36"/>
       <c r="M124" s="36"/>
       <c r="N124" s="36"/>
       <c r="O124" s="36"/>
@@ -8978,9 +8923,7 @@
       <c r="E125" s="41" t="s">
         <v>265</v>
       </c>
-      <c r="F125" s="35">
-        <v>46095</v>
-      </c>
+      <c r="F125" s="35"/>
       <c r="G125" s="35"/>
       <c r="H125" s="35"/>
       <c r="I125" s="40"/>
@@ -8991,7 +8934,7 @@
         <v>506</v>
       </c>
       <c r="L125" s="36" t="s">
-        <v>562</v>
+        <v>555</v>
       </c>
       <c r="M125" s="36"/>
       <c r="N125" s="36"/>
@@ -9023,9 +8966,7 @@
       <c r="E126" s="41" t="s">
         <v>267</v>
       </c>
-      <c r="F126" s="35">
-        <v>46095</v>
-      </c>
+      <c r="F126" s="35"/>
       <c r="G126" s="35"/>
       <c r="H126" s="35"/>
       <c r="I126" s="40"/>
@@ -9036,7 +8977,7 @@
         <v>506</v>
       </c>
       <c r="L126" s="36" t="s">
-        <v>563</v>
+        <v>556</v>
       </c>
       <c r="M126" s="36"/>
       <c r="N126" s="36"/>
@@ -9068,9 +9009,7 @@
       <c r="E127" s="41" t="s">
         <v>269</v>
       </c>
-      <c r="F127" s="35">
-        <v>46095</v>
-      </c>
+      <c r="F127" s="35"/>
       <c r="G127" s="35"/>
       <c r="H127" s="35"/>
       <c r="I127" s="40"/>
@@ -9081,7 +9020,7 @@
         <v>506</v>
       </c>
       <c r="L127" s="36" t="s">
-        <v>564</v>
+        <v>557</v>
       </c>
       <c r="M127" s="36"/>
       <c r="N127" s="36"/>
@@ -9113,9 +9052,7 @@
       <c r="E128" s="41" t="s">
         <v>271</v>
       </c>
-      <c r="F128" s="35">
-        <v>46095</v>
-      </c>
+      <c r="F128" s="35"/>
       <c r="G128" s="35"/>
       <c r="H128" s="35"/>
       <c r="I128" s="40"/>
@@ -9126,7 +9063,7 @@
         <v>506</v>
       </c>
       <c r="L128" s="36" t="s">
-        <v>564</v>
+        <v>557</v>
       </c>
       <c r="M128" s="36"/>
       <c r="N128" s="36"/>
@@ -9158,9 +9095,7 @@
       <c r="E129" s="41" t="s">
         <v>273</v>
       </c>
-      <c r="F129" s="35">
-        <v>46095</v>
-      </c>
+      <c r="F129" s="35"/>
       <c r="G129" s="35"/>
       <c r="H129" s="35"/>
       <c r="I129" s="40"/>
@@ -9171,7 +9106,7 @@
         <v>506</v>
       </c>
       <c r="L129" s="36" t="s">
-        <v>565</v>
+        <v>558</v>
       </c>
       <c r="M129" s="36"/>
       <c r="N129" s="36"/>
@@ -9187,7 +9122,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="130" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A130" s="33">
         <v>169</v>
       </c>
@@ -9207,13 +9142,13 @@
         <v>46095</v>
       </c>
       <c r="G130" s="35" t="s">
-        <v>566</v>
+        <v>559</v>
       </c>
       <c r="H130" s="35" t="s">
-        <v>567</v>
+        <v>560</v>
       </c>
       <c r="I130" s="40" t="s">
-        <v>568</v>
+        <v>561</v>
       </c>
       <c r="J130" s="36" t="s">
         <v>76</v>
@@ -9227,7 +9162,7 @@
         <v>76</v>
       </c>
       <c r="O130" s="36" t="s">
-        <v>569</v>
+        <v>562</v>
       </c>
       <c r="P130" s="36" t="s">
         <v>76</v>
@@ -10473,7 +10408,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="164" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A164" s="33">
         <v>448</v>
       </c>
@@ -10493,13 +10428,13 @@
         <v>46097</v>
       </c>
       <c r="G164" s="35" t="s">
-        <v>570</v>
+        <v>563</v>
       </c>
       <c r="H164" s="35" t="s">
-        <v>571</v>
+        <v>564</v>
       </c>
       <c r="I164" s="40" t="s">
-        <v>572</v>
+        <v>565</v>
       </c>
       <c r="J164" s="36" t="s">
         <v>76</v>
@@ -10520,7 +10455,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="165" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A165" s="33">
         <v>449</v>
       </c>
@@ -10540,13 +10475,13 @@
         <v>46097</v>
       </c>
       <c r="G165" s="35" t="s">
-        <v>573</v>
+        <v>566</v>
       </c>
       <c r="H165" s="35" t="s">
-        <v>574</v>
+        <v>567</v>
       </c>
       <c r="I165" s="40" t="s">
-        <v>575</v>
+        <v>568</v>
       </c>
       <c r="J165" s="36" t="s">
         <v>76</v>
@@ -10953,9 +10888,7 @@
       <c r="E176" s="41" t="s">
         <v>366</v>
       </c>
-      <c r="F176" s="35">
-        <v>46095</v>
-      </c>
+      <c r="F176" s="35"/>
       <c r="G176" s="33"/>
       <c r="H176" s="33"/>
       <c r="I176" s="33"/>
@@ -10966,7 +10899,7 @@
         <v>506</v>
       </c>
       <c r="L176" s="36" t="s">
-        <v>576</v>
+        <v>569</v>
       </c>
       <c r="M176" s="36"/>
       <c r="N176" s="36"/>
@@ -11204,7 +11137,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="183" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A183" s="33">
         <v>468</v>
       </c>
@@ -11224,13 +11157,13 @@
         <v>46097</v>
       </c>
       <c r="G183" s="33" t="s">
-        <v>577</v>
+        <v>570</v>
       </c>
       <c r="H183" s="33" t="s">
-        <v>578</v>
+        <v>571</v>
       </c>
       <c r="I183" s="33" t="s">
-        <v>579</v>
+        <v>572</v>
       </c>
       <c r="J183" s="36" t="s">
         <v>76</v>
@@ -11244,7 +11177,7 @@
         <v>76</v>
       </c>
       <c r="O183" s="36" t="s">
-        <v>580</v>
+        <v>573</v>
       </c>
       <c r="P183" s="36" t="s">
         <v>76</v>
@@ -11256,7 +11189,7 @@
         <v>76</v>
       </c>
       <c r="S183" s="33" t="s">
-        <v>581</v>
+        <v>574</v>
       </c>
       <c r="T183" s="36"/>
       <c r="U183" s="33"/>
@@ -11503,9 +11436,7 @@
       <c r="E190" s="41" t="s">
         <v>394</v>
       </c>
-      <c r="F190" s="35">
-        <v>46097</v>
-      </c>
+      <c r="F190" s="35"/>
       <c r="G190" s="35"/>
       <c r="H190" s="35"/>
       <c r="I190" s="40"/>
@@ -11516,7 +11447,7 @@
         <v>506</v>
       </c>
       <c r="L190" s="36" t="s">
-        <v>558</v>
+        <v>554</v>
       </c>
       <c r="M190" s="36"/>
       <c r="N190" s="36"/>
@@ -16556,6 +16487,11 @@
     <filterColumn colId="2">
       <filters>
         <filter val="RSA"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="9">
+      <filters>
+        <filter val="NO"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -18876,15 +18812,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A92AB09DCDF6014AA0D6826BF29E2C8E" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="58b13f75919cba2dcad85f84b1d5db00">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1e76d14e-d0ce-457c-8343-9b55836d9ead" xmlns:ns3="a56712a3-8dfd-4688-917a-22f0cf513b89" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a3b16ea44285e6579c272a3325f660d0" ns2:_="" ns3:_="">
     <xsd:import namespace="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
@@ -19148,6 +19075,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -19161,14 +19097,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C578C2C-7E0B-429D-96B0-25A2E02D9084}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -19183,6 +19111,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Correzione errori segnalati in data 18/03/2026
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#MYBUSINESSSOLUTIONSXX/MBS/INCARE/1.0/accreditamento-checklist_V8.3.0.xlsx
+++ b/GATEWAY/A1#111#MYBUSINESSSOLUTIONSXX/MBS/INCARE/1.0/accreditamento-checklist_V8.3.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\fse-middleware-accreditamento\GATEWAY\A1#111#MYBUSINESSSOLUTIONSXX\MBS\INCARE\1.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BE27C4D-8639-47F4-A1FA-FD4249F75A51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{072487EA-E57A-4A92-A366-946A51E8DF8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1418" uniqueCount="580">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1418" uniqueCount="577">
   <si>
     <t>COME VALORIZZARE LA CHECKLIST (tab TestCases)</t>
   </si>
@@ -2139,24 +2139,6 @@
     <t>Validazione FSE fallita: [ERRORE-30| L'elemento ClinicalDocument/legalAuthenticator/signatureCode deve essere valorizzato con il codice "S" ]</t>
   </si>
   <si>
-    <t>2026-03-16T11:23:30Z</t>
-  </si>
-  <si>
-    <t>21bad73d64d731ce53028c88940e7bf2</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.10606.20260316120335.d2d1bf47dcc8b68e2e79d565da4dccc6d1124ca447ba93df056c0d9cde8a53cf.9d8643a67c^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
-    <t>2026-03-16T11:25:30Z</t>
-  </si>
-  <si>
-    <t>a45551e7144d83990031ddf07c70b433</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.10606.20260316120335.d2d1bf47dcc8b68e2e79d565da4dccc6d1124ca447ba93df056c0d9cde8a53cf.af81d1af3e^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
-  </si>
-  <si>
     <t>Dato non gestito dal gestionale. Il dottore scrive l’eventuale storia clinica direttamente nel referto</t>
   </si>
   <si>
@@ -2188,6 +2170,15 @@
   </si>
   <si>
     <t>Timeout invio</t>
+  </si>
+  <si>
+    <t>2026-03-19T14:14:30Z</t>
+  </si>
+  <si>
+    <t>258379165692bb139bd29c20134503f1</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.10599.20260319151314.ff023476bbe24b316f4641402f8e9e1605eae930460c7b0d0d6c1190f98c1038.08260593ad^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
 </sst>
 </file>
@@ -4288,7 +4279,7 @@
       </c>
       <c r="B2" s="48"/>
       <c r="C2" s="49" t="s">
-        <v>575</v>
+        <v>569</v>
       </c>
       <c r="D2" s="50"/>
       <c r="F2" s="6"/>
@@ -4316,7 +4307,7 @@
       </c>
       <c r="B3" s="52"/>
       <c r="C3" s="57" t="s">
-        <v>576</v>
+        <v>570</v>
       </c>
       <c r="D3" s="48"/>
       <c r="F3" s="6"/>
@@ -4342,7 +4333,7 @@
       <c r="A4" s="53"/>
       <c r="B4" s="54"/>
       <c r="C4" s="57" t="s">
-        <v>577</v>
+        <v>571</v>
       </c>
       <c r="D4" s="48"/>
       <c r="E4" s="4"/>
@@ -4369,7 +4360,7 @@
       <c r="A5" s="55"/>
       <c r="B5" s="56"/>
       <c r="C5" s="57" t="s">
-        <v>578</v>
+        <v>572</v>
       </c>
       <c r="D5" s="48"/>
       <c r="F5" s="6"/>
@@ -4713,7 +4704,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="15" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="33">
         <v>32</v>
       </c>
@@ -5035,7 +5026,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="23" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="33">
         <v>40</v>
       </c>
@@ -5365,7 +5356,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="31" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="33">
         <v>48</v>
       </c>
@@ -5399,7 +5390,7 @@
         <v>76</v>
       </c>
       <c r="O31" s="36" t="s">
-        <v>579</v>
+        <v>573</v>
       </c>
       <c r="P31" s="36" t="s">
         <v>76</v>
@@ -8536,7 +8527,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="116" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A116" s="33">
         <v>152</v>
       </c>
@@ -8577,7 +8568,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="117" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A117" s="33">
         <v>154</v>
       </c>
@@ -8618,7 +8609,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="118" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A118" s="33">
         <v>155</v>
       </c>
@@ -8659,7 +8650,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="119" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A119" s="33">
         <v>156</v>
       </c>
@@ -8700,7 +8691,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="120" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A120" s="33">
         <v>159</v>
       </c>
@@ -8743,7 +8734,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="121" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A121" s="33">
         <v>160</v>
       </c>
@@ -8784,7 +8775,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="122" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A122" s="33">
         <v>161</v>
       </c>
@@ -8825,7 +8816,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="123" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A123" s="33">
         <v>162</v>
       </c>
@@ -8866,7 +8857,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="124" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A124" s="33">
         <v>163</v>
       </c>
@@ -8907,7 +8898,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="125" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A125" s="33">
         <v>164</v>
       </c>
@@ -8950,7 +8941,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="126" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A126" s="33">
         <v>165</v>
       </c>
@@ -8993,7 +8984,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="127" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A127" s="33">
         <v>166</v>
       </c>
@@ -9036,7 +9027,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="128" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A128" s="33">
         <v>167</v>
       </c>
@@ -9079,7 +9070,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="129" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A129" s="33">
         <v>168</v>
       </c>
@@ -9122,7 +9113,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="130" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A130" s="33">
         <v>169</v>
       </c>
@@ -10408,7 +10399,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="164" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A164" s="33">
         <v>448</v>
       </c>
@@ -10425,16 +10416,16 @@
         <v>342</v>
       </c>
       <c r="F164" s="35">
-        <v>46097</v>
+        <v>46100</v>
       </c>
       <c r="G164" s="35" t="s">
-        <v>563</v>
+        <v>574</v>
       </c>
       <c r="H164" s="35" t="s">
-        <v>564</v>
+        <v>575</v>
       </c>
       <c r="I164" s="40" t="s">
-        <v>565</v>
+        <v>576</v>
       </c>
       <c r="J164" s="36" t="s">
         <v>76</v>
@@ -10455,7 +10446,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="165" spans="1:23" ht="11.1" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:23" ht="11.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A165" s="33">
         <v>449</v>
       </c>
@@ -10472,16 +10463,16 @@
         <v>344</v>
       </c>
       <c r="F165" s="35">
-        <v>46097</v>
+        <v>46100</v>
       </c>
       <c r="G165" s="35" t="s">
-        <v>566</v>
+        <v>574</v>
       </c>
       <c r="H165" s="35" t="s">
-        <v>567</v>
+        <v>575</v>
       </c>
       <c r="I165" s="40" t="s">
-        <v>568</v>
+        <v>576</v>
       </c>
       <c r="J165" s="36" t="s">
         <v>76</v>
@@ -10872,7 +10863,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="176" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A176" s="33">
         <v>461</v>
       </c>
@@ -10899,7 +10890,7 @@
         <v>506</v>
       </c>
       <c r="L176" s="36" t="s">
-        <v>569</v>
+        <v>563</v>
       </c>
       <c r="M176" s="36"/>
       <c r="N176" s="36"/>
@@ -11137,7 +11128,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="183" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A183" s="33">
         <v>468</v>
       </c>
@@ -11157,13 +11148,13 @@
         <v>46097</v>
       </c>
       <c r="G183" s="33" t="s">
-        <v>570</v>
+        <v>564</v>
       </c>
       <c r="H183" s="33" t="s">
-        <v>571</v>
+        <v>565</v>
       </c>
       <c r="I183" s="33" t="s">
-        <v>572</v>
+        <v>566</v>
       </c>
       <c r="J183" s="36" t="s">
         <v>76</v>
@@ -11177,7 +11168,7 @@
         <v>76</v>
       </c>
       <c r="O183" s="36" t="s">
-        <v>573</v>
+        <v>567</v>
       </c>
       <c r="P183" s="36" t="s">
         <v>76</v>
@@ -11189,7 +11180,7 @@
         <v>76</v>
       </c>
       <c r="S183" s="33" t="s">
-        <v>574</v>
+        <v>568</v>
       </c>
       <c r="T183" s="36"/>
       <c r="U183" s="33"/>
@@ -11420,7 +11411,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="190" spans="1:23" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:23" ht="14.25" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A190" s="33">
         <v>475</v>
       </c>
@@ -16491,7 +16482,7 @@
     </filterColumn>
     <filterColumn colId="9">
       <filters>
-        <filter val="NO"/>
+        <filter val="SI"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -18812,6 +18803,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A92AB09DCDF6014AA0D6826BF29E2C8E" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="58b13f75919cba2dcad85f84b1d5db00">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1e76d14e-d0ce-457c-8343-9b55836d9ead" xmlns:ns3="a56712a3-8dfd-4688-917a-22f0cf513b89" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a3b16ea44285e6579c272a3325f660d0" ns2:_="" ns3:_="">
     <xsd:import namespace="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
@@ -19075,15 +19075,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -19097,6 +19088,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C578C2C-7E0B-429D-96B0-25A2E02D9084}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -19111,14 +19110,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Correzione errori del 24/3
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#MYBUSINESSSOLUTIONSXX/MBS/INCARE/1.0/accreditamento-checklist_V8.3.0.xlsx
+++ b/GATEWAY/A1#111#MYBUSINESSSOLUTIONSXX/MBS/INCARE/1.0/accreditamento-checklist_V8.3.0.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\fse-middleware-accreditamento\GATEWAY\A1#111#MYBUSINESSSOLUTIONSXX\MBS\INCARE\1.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B34DD2EB-95D8-498F-926B-70A0D2454E8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A87E556-CD87-45E8-A29F-EFF0E13870DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2172,13 +2172,13 @@
     <t>Timeout invio</t>
   </si>
   <si>
-    <t>2026-03-22T13:46:30Z</t>
-  </si>
-  <si>
-    <t>c10cc6703c83ccfcf92e424b1fd712df</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.10605.20260322144316.807bb47ff5113ba8516f9ea958d19d9a721822c7068a5e67f1be1e83f2a5c1a5.661c1104a8^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>2026-03-30T10:57:30Z</t>
+  </si>
+  <si>
+    <t>7e68f0d423561c3d5b7f176c6b940f0b</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.10608.20260330123901.a0a90e97bcf72056fb4204d69ca85ba22a552eb6f280db28343049d980b8288a.e9f7844480^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
 </sst>
 </file>
@@ -10416,7 +10416,7 @@
         <v>342</v>
       </c>
       <c r="F164" s="35">
-        <v>46103</v>
+        <v>46111</v>
       </c>
       <c r="G164" s="35" t="s">
         <v>574</v>
@@ -10463,7 +10463,7 @@
         <v>344</v>
       </c>
       <c r="F165" s="35">
-        <v>46103</v>
+        <v>46111</v>
       </c>
       <c r="G165" s="35" t="s">
         <v>574</v>
@@ -18803,6 +18803,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A92AB09DCDF6014AA0D6826BF29E2C8E" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="58b13f75919cba2dcad85f84b1d5db00">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1e76d14e-d0ce-457c-8343-9b55836d9ead" xmlns:ns3="a56712a3-8dfd-4688-917a-22f0cf513b89" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a3b16ea44285e6579c272a3325f660d0" ns2:_="" ns3:_="">
     <xsd:import namespace="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
@@ -19066,15 +19075,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -19088,6 +19088,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C578C2C-7E0B-429D-96B0-25A2E02D9084}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -19102,14 +19110,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Costruzione XML CDA2 come da formato suggerito SOGEI
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#MYBUSINESSSOLUTIONSXX/MBS/INCARE/1.0/accreditamento-checklist_V8.3.0.xlsx
+++ b/GATEWAY/A1#111#MYBUSINESSSOLUTIONSXX/MBS/INCARE/1.0/accreditamento-checklist_V8.3.0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\fse-middleware-accreditamento\GATEWAY\A1#111#MYBUSINESSSOLUTIONSXX\MBS\INCARE\1.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A87E556-CD87-45E8-A29F-EFF0E13870DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8766A927-1682-40F4-83D6-4C180DF2BC1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Istruzioni Compilazione" sheetId="1" r:id="rId1"/>
@@ -2172,13 +2172,13 @@
     <t>Timeout invio</t>
   </si>
   <si>
-    <t>2026-03-30T10:57:30Z</t>
-  </si>
-  <si>
-    <t>7e68f0d423561c3d5b7f176c6b940f0b</t>
-  </si>
-  <si>
-    <t>2.16.840.1.113883.2.9.2.120.4.4.10608.20260330123901.a0a90e97bcf72056fb4204d69ca85ba22a552eb6f280db28343049d980b8288a.e9f7844480^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+    <t>2026-03-31T13:06:00Z</t>
+  </si>
+  <si>
+    <t>5b42057475daaf8c38e4b8c6e2e890a9</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.9.2.120.4.4.10605.20260331150316.807bb47ff5113ba8516f9ea958d19d9a721822c7068a5e67f1be1e83f2a5c1a5.2b9e6c98bb^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
   </si>
 </sst>
 </file>
@@ -10416,7 +10416,7 @@
         <v>342</v>
       </c>
       <c r="F164" s="35">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="G164" s="35" t="s">
         <v>574</v>
@@ -10463,7 +10463,7 @@
         <v>344</v>
       </c>
       <c r="F165" s="35">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="G165" s="35" t="s">
         <v>574</v>
@@ -16475,11 +16475,6 @@
     <row r="753" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <autoFilter ref="A9:W245" xr:uid="{00000000-0001-0000-0200-000000000000}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="RSA"/>
-      </filters>
-    </filterColumn>
     <filterColumn colId="9">
       <filters>
         <filter val="SI"/>
@@ -18803,15 +18798,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A92AB09DCDF6014AA0D6826BF29E2C8E" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="58b13f75919cba2dcad85f84b1d5db00">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1e76d14e-d0ce-457c-8343-9b55836d9ead" xmlns:ns3="a56712a3-8dfd-4688-917a-22f0cf513b89" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a3b16ea44285e6579c272a3325f660d0" ns2:_="" ns3:_="">
     <xsd:import namespace="1e76d14e-d0ce-457c-8343-9b55836d9ead"/>
@@ -19075,6 +19061,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -19088,14 +19083,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C578C2C-7E0B-429D-96B0-25A2E02D9084}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -19110,6 +19097,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9413B232-C823-4C2A-B920-858F3EB4F277}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>